<commit_message>
chore: update sunday arrivals workbook
</commit_message>
<xml_diff>
--- a/Sunday_Arrivals.xlsx
+++ b/Sunday_Arrivals.xlsx
@@ -426,16 +426,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Council</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Leader</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>21/06</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>28/06</t>
         </is>
@@ -447,11 +457,16 @@
           <t>Colossians 1</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Isaac Agyeman</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
         <v>143</v>
       </c>
-      <c r="C2" t="n">
-        <v>0</v>
+      <c r="D2" t="n">
+        <v>96</v>
       </c>
     </row>
     <row r="3">
@@ -460,11 +475,16 @@
           <t>Colossians 2</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Edwin Ogoe</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
         <v>83</v>
       </c>
-      <c r="C3" t="n">
-        <v>0</v>
+      <c r="D3" t="n">
+        <v>93</v>
       </c>
     </row>
     <row r="4">
@@ -473,11 +493,16 @@
           <t>Colossians 3</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Nathan Kudowor</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
         <v>64</v>
       </c>
-      <c r="C4" t="n">
-        <v>0</v>
+      <c r="D4" t="n">
+        <v>43</v>
       </c>
     </row>
     <row r="5">
@@ -486,11 +511,11 @@
           <t>Colossians Total</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="C5" t="n">
         <v>290</v>
       </c>
-      <c r="C5" t="n">
-        <v>0</v>
+      <c r="D5" t="n">
+        <v>232</v>
       </c>
     </row>
     <row r="7">
@@ -499,11 +524,16 @@
           <t>Galatians 1</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Isaac Agyeman</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
         <v>38</v>
       </c>
-      <c r="C7" t="n">
-        <v>0</v>
+      <c r="D7" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="8">
@@ -512,11 +542,16 @@
           <t>Galatians 2</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Richmond Annan</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
         <v>158</v>
       </c>
-      <c r="C8" t="n">
-        <v>0</v>
+      <c r="D8" t="n">
+        <v>128</v>
       </c>
     </row>
     <row r="9">
@@ -525,10 +560,15 @@
           <t>Galatians 2 (Hold)</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>0</v>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Edwin Ogoe</t>
+        </is>
       </c>
       <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -538,11 +578,16 @@
           <t>Galatians 4</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Eric Boachie Yiadom</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
         <v>100</v>
       </c>
-      <c r="C10" t="n">
-        <v>0</v>
+      <c r="D10" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="11">
@@ -551,11 +596,16 @@
           <t>Galatians 5</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Michael Oteng</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
         <v>157</v>
       </c>
-      <c r="C11" t="n">
-        <v>0</v>
+      <c r="D11" t="n">
+        <v>116</v>
       </c>
     </row>
     <row r="12">
@@ -564,11 +614,16 @@
           <t>Galatians 8</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Caleb Osei-Kofi</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
         <v>137</v>
       </c>
-      <c r="C12" t="n">
-        <v>0</v>
+      <c r="D12" t="n">
+        <v>90</v>
       </c>
     </row>
     <row r="13">
@@ -577,11 +632,16 @@
           <t>Galatians 9</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Divine Olubakinde</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
         <v>87</v>
       </c>
-      <c r="C13" t="n">
-        <v>0</v>
+      <c r="D13" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="14">
@@ -590,11 +650,11 @@
           <t>Galatians Total</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="C14" t="n">
         <v>677</v>
       </c>
-      <c r="C14" t="n">
-        <v>0</v>
+      <c r="D14" t="n">
+        <v>507</v>
       </c>
     </row>
     <row r="16">
@@ -603,11 +663,16 @@
           <t>Galatians 3</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Joseph Teye</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
         <v>99</v>
       </c>
-      <c r="C16" t="n">
-        <v>0</v>
+      <c r="D16" t="n">
+        <v>79</v>
       </c>
     </row>
     <row r="17">
@@ -616,11 +681,16 @@
           <t>Galatians 6 A</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Nana Kofi Danso-Mensah</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
         <v>121</v>
       </c>
-      <c r="C17" t="n">
-        <v>0</v>
+      <c r="D17" t="n">
+        <v>94</v>
       </c>
     </row>
     <row r="18">
@@ -629,11 +699,16 @@
           <t>Galatians 7</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Albert Gillies Heward-Mills</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
         <v>206</v>
       </c>
-      <c r="C18" t="n">
-        <v>0</v>
+      <c r="D18" t="n">
+        <v>144</v>
       </c>
     </row>
     <row r="19">
@@ -642,11 +717,11 @@
           <t>Jesus Night Total</t>
         </is>
       </c>
-      <c r="B19" t="n">
+      <c r="C19" t="n">
         <v>426</v>
       </c>
-      <c r="C19" t="n">
-        <v>0</v>
+      <c r="D19" t="n">
+        <v>317</v>
       </c>
     </row>
     <row r="21">
@@ -655,11 +730,11 @@
           <t>Grand Total</t>
         </is>
       </c>
-      <c r="B21" t="n">
+      <c r="C21" t="n">
         <v>1393</v>
       </c>
-      <c r="C21" t="n">
-        <v>0</v>
+      <c r="D21" t="n">
+        <v>1056</v>
       </c>
     </row>
   </sheetData>
@@ -713,7 +788,7 @@
         <v>6</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
@@ -731,7 +806,7 @@
         <v>6</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -749,7 +824,7 @@
         <v>16</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
@@ -785,7 +860,7 @@
         <v>36</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7">
@@ -803,7 +878,7 @@
         <v>7</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
@@ -839,7 +914,7 @@
         <v>8</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10">
@@ -857,7 +932,7 @@
         <v>26</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11">
@@ -875,7 +950,7 @@
         <v>28</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12">
@@ -893,15 +968,20 @@
         <v>15</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
       <c r="C13" t="n">
         <v>157</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -955,7 +1035,7 @@
         <v>14</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3">
@@ -973,7 +1053,7 @@
         <v>16</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -991,7 +1071,7 @@
         <v>14</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -1009,7 +1089,7 @@
         <v>11</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -1027,7 +1107,7 @@
         <v>14</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
@@ -1045,7 +1125,7 @@
         <v>16</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8">
@@ -1063,7 +1143,7 @@
         <v>26</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9">
@@ -1081,7 +1161,7 @@
         <v>3</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -1099,15 +1179,20 @@
         <v>7</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
       <c r="C11" t="n">
         <v>121</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -1161,7 +1246,7 @@
         <v>11</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
@@ -1215,7 +1300,7 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -1233,7 +1318,7 @@
         <v>7</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -1269,7 +1354,7 @@
         <v>35</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9">
@@ -1287,7 +1372,7 @@
         <v>31</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10">
@@ -1305,7 +1390,7 @@
         <v>4</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
@@ -1323,7 +1408,7 @@
         <v>54</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -1341,7 +1426,7 @@
         <v>14</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13">
@@ -1359,7 +1444,7 @@
         <v>29</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14">
@@ -1377,7 +1462,7 @@
         <v>12</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15">
@@ -1395,7 +1480,7 @@
         <v>8</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16">
@@ -1417,11 +1502,16 @@
       </c>
     </row>
     <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
       <c r="C17" t="n">
         <v>206</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -1475,7 +1565,7 @@
         <v>17</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -1493,7 +1583,7 @@
         <v>36</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4">
@@ -1529,7 +1619,7 @@
         <v>20</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
@@ -1547,7 +1637,7 @@
         <v>8</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7">
@@ -1565,7 +1655,7 @@
         <v>41</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8">
@@ -1583,15 +1673,20 @@
         <v>15</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
       <c r="C9" t="n">
         <v>137</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -1645,7 +1740,7 @@
         <v>24</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3">
@@ -1663,7 +1758,7 @@
         <v>20</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -1681,7 +1776,7 @@
         <v>13</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -1717,7 +1812,7 @@
         <v>9</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -1735,7 +1830,7 @@
         <v>15</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -1753,15 +1848,20 @@
         <v>6</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
       <c r="C9" t="n">
         <v>87</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -1833,7 +1933,7 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -1851,7 +1951,7 @@
         <v>28</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
@@ -1869,7 +1969,7 @@
         <v>15</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6">
@@ -1905,7 +2005,7 @@
         <v>14</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -1923,7 +2023,7 @@
         <v>22</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9">
@@ -1941,7 +2041,7 @@
         <v>12</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
@@ -1959,7 +2059,7 @@
         <v>12</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
@@ -1977,7 +2077,7 @@
         <v>5</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12">
@@ -1995,15 +2095,20 @@
         <v>14</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
       <c r="C13" t="n">
         <v>143</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -2111,7 +2216,7 @@
         <v>52</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6">
@@ -2129,7 +2234,7 @@
         <v>16</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7">
@@ -2183,15 +2288,20 @@
         <v>15</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
       <c r="C10" t="n">
         <v>83</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -2245,7 +2355,7 @@
         <v>13</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3">
@@ -2263,7 +2373,7 @@
         <v>11</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -2281,7 +2391,7 @@
         <v>20</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
@@ -2317,15 +2427,20 @@
         <v>20</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
       <c r="C7" t="n">
         <v>64</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -2379,7 +2494,7 @@
         <v>20</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3">
@@ -2397,15 +2512,20 @@
         <v>18</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
       <c r="C4" t="n">
         <v>38</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -2477,7 +2597,7 @@
         <v>18</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4">
@@ -2495,7 +2615,7 @@
         <v>22</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5">
@@ -2513,7 +2633,7 @@
         <v>16</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -2531,7 +2651,7 @@
         <v>36</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7">
@@ -2549,7 +2669,7 @@
         <v>12</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8">
@@ -2567,7 +2687,7 @@
         <v>31</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9">
@@ -2585,7 +2705,7 @@
         <v>15</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
@@ -2603,15 +2723,20 @@
         <v>8</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
       <c r="C11" t="n">
         <v>158</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -2651,6 +2776,11 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
       <c r="C2" t="n">
         <v>0</v>
       </c>
@@ -2709,7 +2839,7 @@
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -2745,7 +2875,7 @@
         <v>12</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -2763,7 +2893,7 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
@@ -2781,7 +2911,7 @@
         <v>37</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7">
@@ -2799,15 +2929,20 @@
         <v>47</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
       <c r="C8" t="n">
         <v>99</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -2861,7 +2996,7 @@
         <v>27</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3">
@@ -2879,7 +3014,7 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -2897,7 +3032,7 @@
         <v>25</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5">
@@ -2915,7 +3050,7 @@
         <v>48</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6">
@@ -2937,11 +3072,16 @@
       </c>
     </row>
     <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
       <c r="C7" t="n">
         <v>100</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>